<commit_message>
xgb implementation ->  ACC up to 77%
</commit_message>
<xml_diff>
--- a/output/all_predictions.xlsx
+++ b/output/all_predictions.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.8590492246463678</v>
+        <v>0.859049225</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.6312136768269763</v>
+        <v>0.631213677</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.6416335120899616</v>
+        <v>0.641633512</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.654368185331398</v>
+        <v>0.654368185</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.8596300648781309</v>
+        <v>0.8596300650000001</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6543681885696864</v>
+        <v>0.654368189</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.8470377267810785</v>
+        <v>0.847037727</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.6468508019870481</v>
+        <v>0.646850802</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.749628072689052</v>
+        <v>0.749628073</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.2970138352607768</v>
+        <v>0.297013835</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -805,29 +805,31 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.3942169236533269</v>
+        <v>0.730219433</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>22500964</v>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>22500968.0</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -836,29 +838,31 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chicago Bulls</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.730219433274207</v>
+        <v>0.418848648</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>22500968</v>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>22500965.0</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -867,29 +871,31 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.5861016864721887</v>
+        <v>0.394216924</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>22500966</v>
+          <t>Houston Rockets</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>22500964.0</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -898,29 +904,31 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dallas Mavericks</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.4188486482337365</v>
+        <v>0.586101686</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>22500965</v>
+          <t>Minnesota Timberwolves</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>22500966.0</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -929,29 +937,31 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Indiana Pacers</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.3162462892533334</v>
+        <v>0.695789952</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>22500962</v>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>22500961.0</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -960,29 +970,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.695789951599302</v>
+        <v>0.569645035</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>22500961</v>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>22500967.0</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -991,29 +1003,31 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.4189104333098274</v>
+        <v>0.316246289</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>22500963</v>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>22500962.0</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1022,29 +1036,248 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Utah Jazz</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.5696450348251237</v>
+        <v>0.418910433</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>22500967</v>
+          <t>Toronto Raptors</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>22500963.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Brooklyn Nets</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5775021314620972</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>22500969</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Milwaukee Bucks</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.8429240584373474</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>22500970</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.6524375677108765</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>22500973</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Washington Wizards</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.8574886322021484</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>22500971</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Miami Heat</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.4993022978305817</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>22500972</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.6525467038154602</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>22500974</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sacramento Kings</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.5777215957641602</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sacramento Kings</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>22500975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Acc 16.03 von 71% mit 5 von 7 treffer
</commit_message>
<xml_diff>
--- a/output/all_predictions.xlsx
+++ b/output/all_predictions.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,48 +417,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Home Team</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Away Team</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Predicted Winner</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>probability_home_win</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Actual Winner</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>gameId</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -503,7 +491,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -536,7 +524,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -569,7 +557,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -602,7 +590,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -635,7 +623,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -661,14 +649,10 @@
           <t>Detroit Pistons</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -701,7 +685,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -734,7 +718,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -767,7 +751,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>46093</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -800,484 +784,746 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>Toronto Raptors</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Phoenix Suns</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Phoenix Suns</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.418910433</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Toronto Raptors</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>22500963.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Utah Jazz</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.569645035</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>22500967.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Memphis Grizzlies</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.695789952</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>22500961.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Indiana Pacers</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.316246289</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>22500962.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Houston Rockets</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>New Orleans Pelicans</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>New Orleans Pelicans</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.394216924</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Houston Rockets</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>22500964.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Dallas Mavericks</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.418848648</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>22500965.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>LA Clippers</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Chicago Bulls</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>LA Clippers</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E18" t="n">
         <v>0.730219433</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>LA Clippers</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>22500968.0</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Golden State Warriors</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Minnesota Timberwolves</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Golden State Warriors</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.586101686</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Minnesota Timberwolves</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>22500966.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sacramento Kings</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5777215957641602</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Sacramento Kings</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>22500975.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Miami Heat</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.4993022978305817</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>22500972.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Washington Wizards</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.8574886322021484</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>22500971.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.6525467038154602</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>22500974.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Milwaukee Bucks</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.8429240584373474</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>22500970.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Brooklyn Nets</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.5775021314620972</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>22500969.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>46095</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.6524375677108765</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>22500973.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Brooklyn Nets</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Brooklyn Nets</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.5038461685180664</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>22500985</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>New Orleans Pelicans</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>Dallas Mavericks</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Cleveland Cavaliers</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Cleveland Cavaliers</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>0.418848648</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Cleveland Cavaliers</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>22500965.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>New Orleans Pelicans</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.7718399167060852</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>New Orleans Pelicans</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>22500988</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Phoenix Suns</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.6628966331481934</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>22500986</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Washington Wizards</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Golden State Warriors</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Golden State Warriors</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.222200021147728</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Golden State Warriors</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>22500984</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>Houston Rockets</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>New Orleans Pelicans</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>New Orleans Pelicans</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>0.394216924</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Houston Rockets</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>22500964.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Golden State Warriors</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Minnesota Timberwolves</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Golden State Warriors</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>0.586101686</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Minnesota Timberwolves</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>22500966.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Detroit Pistons</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.4305817782878876</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>22500989</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>LA Clippers</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.5851534008979797</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>22500990</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.5979579091072083</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>22500983</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Chicago Bulls</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>Memphis Grizzlies</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Detroit Pistons</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>0.695789952</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Detroit Pistons</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>22500961.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Portland Trail Blazers</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Utah Jazz</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Portland Trail Blazers</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>0.569645035</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Portland Trail Blazers</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>22500967.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Indiana Pacers</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>New York Knicks</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>New York Knicks</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>0.316246289</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>New York Knicks</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>22500962.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>46094</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Toronto Raptors</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Phoenix Suns</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Phoenix Suns</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>0.418910433</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Toronto Raptors</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>22500963.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Philadelphia 76ers</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Brooklyn Nets</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Philadelphia 76ers</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>0.5775021314620972</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Philadelphia 76ers</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>22500969</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Atlanta Hawks</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Milwaukee Bucks</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Atlanta Hawks</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>0.8429240584373474</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Atlanta Hawks</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>22500970</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>San Antonio Spurs</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Charlotte Hornets</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>San Antonio Spurs</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>0.6524375677108765</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>San Antonio Spurs</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>22500973</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Boston Celtics</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Washington Wizards</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Boston Celtics</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>0.8574886322021484</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Boston Celtics</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>22500971</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Miami Heat</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Orlando Magic</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Orlando Magic</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>0.4993022978305817</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Orlando Magic</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>22500972</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Los Angeles Lakers</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Denver Nuggets</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Los Angeles Lakers</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>0.6525467038154602</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Los Angeles Lakers</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>22500974</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>46095</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>LA Clippers</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Sacramento Kings</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>LA Clippers</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>0.5777215957641602</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Sacramento Kings</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>22500975</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Chicago Bulls</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.6791099905967712</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Chicago Bulls</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>22500987</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vorhersagen für gestern 100%
</commit_message>
<xml_diff>
--- a/output/all_predictions.xlsx
+++ b/output/all_predictions.xlsx
@@ -789,30 +789,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.418910433</v>
+        <v>0.316246289</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>22500963.0</t>
+          <t>22500962.0</t>
         </is>
       </c>
     </row>
@@ -822,30 +822,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Utah Jazz</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.569645035</v>
+        <v>0.695789952</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>22500967.0</t>
+          <t>22500961.0</t>
         </is>
       </c>
     </row>
@@ -855,30 +855,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.695789952</v>
+        <v>0.418910433</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>22500961.0</t>
+          <t>22500963.0</t>
         </is>
       </c>
     </row>
@@ -888,30 +888,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Indiana Pacers</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.316246289</v>
+        <v>0.569645035</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>22500962.0</t>
+          <t>22500967.0</t>
         </is>
       </c>
     </row>
@@ -921,30 +921,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.394216924</v>
+        <v>0.418848648</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>22500964.0</t>
+          <t>22500965.0</t>
         </is>
       </c>
     </row>
@@ -954,30 +954,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dallas Mavericks</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Chicago Bulls</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.418848648</v>
+        <v>0.730219433</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>22500965.0</t>
+          <t>22500968.0</t>
         </is>
       </c>
     </row>
@@ -987,30 +987,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Chicago Bulls</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.730219433</v>
+        <v>0.586101686</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>22500968.0</t>
+          <t>22500966.0</t>
         </is>
       </c>
     </row>
@@ -1020,30 +1020,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.586101686</v>
+        <v>0.394216924</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>22500966.0</t>
+          <t>22500964.0</t>
         </is>
       </c>
     </row>
@@ -1053,30 +1053,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.5777215957641602</v>
+        <v>0.652546704</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>22500975.0</t>
+          <t>22500974.0</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.4993022978305817</v>
+        <v>0.499302298</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.8574886322021484</v>
+        <v>0.857488632</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1152,30 +1152,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Denver Nuggets</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.6525467038154602</v>
+        <v>0.5777215959999999</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>22500974.0</t>
+          <t>22500975.0</t>
         </is>
       </c>
     </row>
@@ -1185,30 +1185,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Milwaukee Bucks</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.8429240584373474</v>
+        <v>0.652437568</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>22500970.0</t>
+          <t>22500973.0</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.5775021314620972</v>
+        <v>0.577502131</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1251,30 +1251,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.6524375677108765</v>
+        <v>0.842924058</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>22500973.0</t>
+          <t>22500970.0</t>
         </is>
       </c>
     </row>
@@ -1284,29 +1284,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Brooklyn Nets</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brooklyn Nets</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.5038461685180664</v>
+        <v>0.1696883141994476</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>22500985</v>
+        <v>22500984</v>
       </c>
     </row>
     <row r="28">
@@ -1315,29 +1315,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dallas Mavericks</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.7718399167060852</v>
+        <v>0.3228119611740112</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>22500988</v>
+        <v>22500989</v>
       </c>
     </row>
     <row r="29">
@@ -1346,29 +1346,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.6628966331481934</v>
+        <v>0.4246545135974884</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>22500986</v>
+        <v>22500990</v>
       </c>
     </row>
     <row r="30">
@@ -1377,29 +1377,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Washington Wizards</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.222200021147728</v>
+        <v>0.628429651260376</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>22500984</v>
+        <v>22500983</v>
       </c>
     </row>
     <row r="31">
@@ -1408,29 +1408,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Brooklyn Nets</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.4305817782878876</v>
+        <v>0.2950863242149353</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>22500989</v>
+        <v>22500985</v>
       </c>
     </row>
     <row r="32">
@@ -1439,29 +1439,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.5851534008979797</v>
+        <v>0.8141456246376038</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>22500990</v>
+        <v>22500988</v>
       </c>
     </row>
     <row r="33">
@@ -1470,29 +1470,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.5979579091072083</v>
+        <v>0.7310704588890076</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>22500983</v>
+        <v>22500986</v>
       </c>
     </row>
     <row r="34">
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.6791099905967712</v>
+        <v>0.7086217999458313</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
17.03 ACC von 88%
</commit_message>
<xml_diff>
--- a/output/all_predictions.xlsx
+++ b/output/all_predictions.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -789,30 +789,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Indiana Pacers</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.316246289</v>
+        <v>0.569645035</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>22500962.0</t>
+          <t>22500967.0</t>
         </is>
       </c>
     </row>
@@ -888,30 +888,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Utah Jazz</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.569645035</v>
+        <v>0.316246289</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>22500967.0</t>
+          <t>22500962.0</t>
         </is>
       </c>
     </row>
@@ -921,30 +921,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dallas Mavericks</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.418848648</v>
+        <v>0.394216924</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>22500965.0</t>
+          <t>22500964.0</t>
         </is>
       </c>
     </row>
@@ -1020,30 +1020,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.394216924</v>
+        <v>0.418848648</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>22500964.0</t>
+          <t>22500965.0</t>
         </is>
       </c>
     </row>
@@ -1086,30 +1086,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Miami Heat</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.499302298</v>
+        <v>0.5777215959999999</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>22500972.0</t>
+          <t>22500975.0</t>
         </is>
       </c>
     </row>
@@ -1119,30 +1119,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Washington Wizards</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.857488632</v>
+        <v>0.499302298</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>22500971.0</t>
+          <t>22500972.0</t>
         </is>
       </c>
     </row>
@@ -1152,30 +1152,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.5777215959999999</v>
+        <v>0.652437568</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>22500975.0</t>
+          <t>22500973.0</t>
         </is>
       </c>
     </row>
@@ -1185,30 +1185,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.652437568</v>
+        <v>0.842924058</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>22500973.0</t>
+          <t>22500970.0</t>
         </is>
       </c>
     </row>
@@ -1251,30 +1251,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Milwaukee Bucks</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.842924058</v>
+        <v>0.857488632</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>22500970.0</t>
+          <t>22500971.0</t>
         </is>
       </c>
     </row>
@@ -1284,29 +1284,31 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Washington Wizards</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.1696883141994476</v>
+        <v>0.814145625</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Golden State Warriors</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>22500984</v>
+          <t>New Orleans Pelicans</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>22500988.0</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1315,29 +1317,31 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Boston Celtics</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.3228119611740112</v>
+        <v>0.731070459</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>22500989</v>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>22500986.0</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1346,29 +1350,31 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>Golden State Warriors</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.4246545135974884</v>
+        <v>0.169688314</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
-        </is>
-      </c>
-      <c r="G29" t="n">
-        <v>22500990</v>
+          <t>Golden State Warriors</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>22500984.0</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1377,29 +1383,31 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
+          <t>Los Angeles Lakers</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.628429651260376</v>
+        <v>0.322811961</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Atlanta Hawks</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>22500983</v>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>22500989.0</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1408,29 +1416,31 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Brooklyn Nets</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
+          <t>San Antonio Spurs</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.2950863242149353</v>
+        <v>0.424654514</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Portland Trail Blazers</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>22500985</v>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>22500990.0</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1439,29 +1449,31 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dallas Mavericks</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.8141456246376038</v>
+        <v>0.628429651</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>22500988</v>
+          <t>Atlanta Hawks</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>22500983.0</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1470,29 +1482,31 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>Brooklyn Nets</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>Portland Trail Blazers</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.7310704588890076</v>
+        <v>0.295086324</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>22500986</v>
+          <t>Portland Trail Blazers</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>22500985.0</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1515,15 +1529,265 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.7086217999458313</v>
+        <v>0.7086218</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>Chicago Bulls</t>
         </is>
       </c>
-      <c r="G34" t="n">
-        <v>22500987</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>22500987.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Washington Wizards</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0.1621145457029343</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Detroit Pistons</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>22500993</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Miami Heat</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.5457360744476318</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Charlotte Hornets</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>22500991</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Indiana Pacers</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.7550305724143982</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>22500994</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sacramento Kings</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.3026701211929321</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>22500998</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Milwaukee Bucks</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.3743271231651306</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Cleveland Cavaliers</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>22500995</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Minnesota Timberwolves</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Phoenix Suns</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Phoenix Suns</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.4343498349189758</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Minnesota Timberwolves</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>22500996</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Orlando Magic</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Oklahoma City Thunder</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Oklahoma City Thunder</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.2116377651691437</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Oklahoma City Thunder</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>22500992</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Philadelphia 76ers</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.6574461460113525</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>22500997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>